<commit_message>
Add BP Pharma, CLD Surgical, MP Enterprise invoice data to rate card; rebuild bills
Rate card updates:
- SL83 Plain Sheet: MRP=₹200, Cost=₹65 (BP Pharma #248/#288 PLAIN SHEET D301) — MRP was missing
- SL85 Gypsona 4" POP: MRP=₹19.92, Cost=₹11.58 per roll (BP Pharma #288, 12/pack)
- SL65 Gloves 7.0: Cost updated to ₹22 (BP Pharma SURGICARE 7.0)
- SL49 Uro Bag: Cost updated to ₹40.50 (CLD Surgical #270)
- SL50 Foley's 16Fr: Cost updated to ₹126.50 (BP Pharma #248)
- SL119: NS 3000ml — MRP=₹698.44, Cost=₹133.33
- SL120: Gypsona 6" POP — MRP=₹24.92, Cost=₹14.62
- SL121-127: TUR Set, C-Arm Cover, LMA 3.0/4.0, ET Tube No.6, RAE Nasal, Romo Bougie

Bills: Rebuilt — Plain Sheet (SL83) orange flags removed from Pt28 and Pt35

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_June2026_Bills.xlsx
+++ b/BKAditya_June2026_Bills.xlsx
@@ -4416,17 +4416,16 @@
       <c r="C22" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>⚠ ENTER MRP</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="25" t="inlineStr">
-        <is>
-          <t>SL83 — MRP missing, enter manually</t>
+      <c r="D22" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="E22" s="21">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>SL83 / Plain Sheet (OT Draping)</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4441,7 @@
       </c>
       <c r="F23" s="25" t="inlineStr">
         <is>
-          <t>⚠ 2 item(s) need MRP — total partial</t>
+          <t>⚠ 1 item(s) need MRP — total partial</t>
         </is>
       </c>
     </row>
@@ -8819,17 +8818,16 @@
       <c r="C28" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="D28" s="23" t="inlineStr">
-        <is>
-          <t>⚠ ENTER MRP</t>
-        </is>
-      </c>
-      <c r="E28" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="25" t="inlineStr">
-        <is>
-          <t>SL83 — MRP missing, enter manually</t>
+      <c r="D28" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="E28" s="21">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>SL83 / Plain Sheet (OT Draping)</t>
         </is>
       </c>
     </row>
@@ -9195,7 +9193,7 @@
       </c>
       <c r="F43" s="25" t="inlineStr">
         <is>
-          <t>⚠ 2 item(s) need MRP — total partial</t>
+          <t>⚠ 1 item(s) need MRP — total partial</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pt30 Shankari Chakraborty: add items from OT sheet + 2 ward indents + dress changes
Previously only had partial items. Now includes all 3 documents:
- OT sheet (08/06): Spinocaine, Gypsona x2, sutures, cap+mask x6, syringes
- Ward indent #82 (08/06): Moly sheet, Foley 16Fr, Uro bag, Neomol x7, full fluids
- Ward indent #84 (12/06): PCM 100ml x3, Cetil x2, Tramadol x2
- Dressing changes (10/6+13/6): Gamji Roll x3, Gauze updated 12→28, Gloves 6.5 x3
Total items: 21 → 32

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_June2026_Bills.xlsx
+++ b/BKAditya_June2026_Bills.xlsx
@@ -5364,14 +5364,14 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>NS 500ml</t>
+          <t>Inj. Anawin Heavy 0.75% (Spinocaine)</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>39.05</v>
+        <v>31.47</v>
       </c>
       <c r="E12" s="21">
         <f>C12*D12</f>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="F12" s="22" t="inlineStr">
         <is>
-          <t>SL1 / NS 500ml — Normal Saline</t>
+          <t>SL7 / Inj. Anawin Heavy 0.75%/4ml (Bupiva</t>
         </is>
       </c>
     </row>
@@ -5389,14 +5389,14 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>NS 100ml</t>
+          <t>IV Set</t>
         </is>
       </c>
       <c r="C13" s="20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D13" s="21" t="n">
-        <v>21</v>
+        <v>201</v>
       </c>
       <c r="E13" s="21">
         <f>C13*D13</f>
@@ -5404,7 +5404,7 @@
       </c>
       <c r="F13" s="22" t="inlineStr">
         <is>
-          <t>SL3 / NS 100ml — Normal Saline 100ml</t>
+          <t>SL44 / IV Set / Sangoflex</t>
         </is>
       </c>
     </row>
@@ -5418,7 +5418,7 @@
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="21" t="n">
         <v>202.55</v>
@@ -5439,14 +5439,14 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Inj. Ondem</t>
+          <t>Easyfix</t>
         </is>
       </c>
       <c r="C15" s="20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>12.72</v>
+        <v>900</v>
       </c>
       <c r="E15" s="21">
         <f>C15*D15</f>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="F15" s="22" t="inlineStr">
         <is>
-          <t>SL29 / Inj. Ondem/Zofer/Zofar (Ondansetron</t>
+          <t>SL48 / Easyfix (Adhesive Film Dressing)</t>
         </is>
       </c>
     </row>
@@ -5464,14 +5464,14 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Inj. Pan IV</t>
+          <t>Syringe 10ml</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>53.9</v>
+        <v>20</v>
       </c>
       <c r="E16" s="21">
         <f>C16*D16</f>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t>SL33 / Inj. Pan 40 / Pantocid (Pantoprazol</t>
+          <t>SL56 / Syringe 10cc / 10ml</t>
         </is>
       </c>
     </row>
@@ -5489,14 +5489,14 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Inj. Xone 1g</t>
+          <t>Syringe 5ml</t>
         </is>
       </c>
       <c r="C17" s="20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D17" s="21" t="n">
-        <v>66.64</v>
+        <v>10.23</v>
       </c>
       <c r="E17" s="21">
         <f>C17*D17</f>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="F17" s="22" t="inlineStr">
         <is>
-          <t>SL16 / Inj. Xone/Monocef 1g (Ceftriaxone)</t>
+          <t>SL57 / Syringe 5cc / 5ml</t>
         </is>
       </c>
     </row>
@@ -5514,14 +5514,14 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>IV Set</t>
+          <t>Syringe 2ml</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
         <v>2</v>
       </c>
       <c r="D18" s="21" t="n">
-        <v>201</v>
+        <v>6.04</v>
       </c>
       <c r="E18" s="21">
         <f>C18*D18</f>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="F18" s="22" t="inlineStr">
         <is>
-          <t>SL44 / IV Set / Sangoflex</t>
+          <t>SL58 / Syringe 2cc / 2ml</t>
         </is>
       </c>
     </row>
@@ -5539,14 +5539,14 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>RL 500ml</t>
+          <t>D. Water 10ml</t>
         </is>
       </c>
       <c r="C19" s="20" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D19" s="21" t="n">
-        <v>63.3</v>
+        <v>3.24</v>
       </c>
       <c r="E19" s="21">
         <f>C19*D19</f>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="F19" s="22" t="inlineStr">
         <is>
-          <t>SL4 / RL 500ml — Ringer's Lactate</t>
+          <t>SL59 / D. Water 10ml (Sterile Water)</t>
         </is>
       </c>
     </row>
@@ -5564,14 +5564,14 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Easyfix</t>
+          <t>Gypsona POP Bandage 4"</t>
         </is>
       </c>
       <c r="C20" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="21" t="n">
-        <v>900</v>
+        <v>19.92</v>
       </c>
       <c r="E20" s="21">
         <f>C20*D20</f>
@@ -5579,7 +5579,7 @@
       </c>
       <c r="F20" s="22" t="inlineStr">
         <is>
-          <t>SL48 / Easyfix (Adhesive Film Dressing)</t>
+          <t>SL85 / Gypsona POP Bandage 40G</t>
         </is>
       </c>
     </row>
@@ -5589,14 +5589,14 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Inj. Diclofenac AQ (Justin)</t>
+          <t>Suture Ethilon 2-0</t>
         </is>
       </c>
       <c r="C21" s="20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21" s="21" t="n">
-        <v>23.8</v>
+        <v>277</v>
       </c>
       <c r="E21" s="21">
         <f>C21*D21</f>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="F21" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">SL22 / Inj. Dynapar/Justin AQ (Diclofenac </t>
+          <t>SL77 / Suture Ethilon 2-0 / SN9336TFP</t>
         </is>
       </c>
     </row>
@@ -5614,14 +5614,14 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Syringe 10ml</t>
+          <t>Suture Vicryl 1</t>
         </is>
       </c>
       <c r="C22" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="21" t="n">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="E22" s="21">
         <f>C22*D22</f>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="F22" s="22" t="inlineStr">
         <is>
-          <t>SL56 / Syringe 10cc / 10ml</t>
+          <t>SL78 / Suture Vicryl 1 (2421)</t>
         </is>
       </c>
     </row>
@@ -5639,22 +5639,23 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Syringe 5ml</t>
+          <t>Cap + Mask Set</t>
         </is>
       </c>
       <c r="C23" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" s="21" t="n">
-        <v>10.23</v>
-      </c>
-      <c r="E23" s="21">
-        <f>C23*D23</f>
-        <v/>
-      </c>
-      <c r="F23" s="22" t="inlineStr">
-        <is>
-          <t>SL57 / Syringe 5cc / 5ml</t>
+        <v>6</v>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>⚠ ENTER MRP</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="25" t="inlineStr">
+        <is>
+          <t>SL86 — MRP missing, enter manually</t>
         </is>
       </c>
     </row>
@@ -5664,14 +5665,14 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Syringe 2ml</t>
+          <t>NS 500ml</t>
         </is>
       </c>
       <c r="C24" s="20" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D24" s="21" t="n">
-        <v>6.04</v>
+        <v>39.05</v>
       </c>
       <c r="E24" s="21">
         <f>C24*D24</f>
@@ -5679,7 +5680,7 @@
       </c>
       <c r="F24" s="22" t="inlineStr">
         <is>
-          <t>SL58 / Syringe 2cc / 2ml</t>
+          <t>SL1 / NS 500ml — Normal Saline</t>
         </is>
       </c>
     </row>
@@ -5689,14 +5690,14 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>D. Water 10ml</t>
+          <t>NS 100ml</t>
         </is>
       </c>
       <c r="C25" s="20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="21" t="n">
-        <v>3.24</v>
+        <v>21</v>
       </c>
       <c r="E25" s="21">
         <f>C25*D25</f>
@@ -5704,7 +5705,7 @@
       </c>
       <c r="F25" s="22" t="inlineStr">
         <is>
-          <t>SL59 / D. Water 10ml (Sterile Water)</t>
+          <t>SL3 / NS 100ml — Normal Saline 100ml</t>
         </is>
       </c>
     </row>
@@ -5714,14 +5715,14 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>Gloves 6.5 Sterile</t>
+          <t>RL 500ml</t>
         </is>
       </c>
       <c r="C26" s="20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" s="21" t="n">
-        <v>91</v>
+        <v>63.3</v>
       </c>
       <c r="E26" s="21">
         <f>C26*D26</f>
@@ -5729,7 +5730,7 @@
       </c>
       <c r="F26" s="22" t="inlineStr">
         <is>
-          <t>SL65 / Gloves 7.0 (Sterile Surgical)</t>
+          <t>SL4 / RL 500ml — Ringer's Lactate</t>
         </is>
       </c>
     </row>
@@ -5739,14 +5740,14 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Gauze Pieces (Sterile)</t>
+          <t>Moli/Mackintosh Sheet</t>
         </is>
       </c>
       <c r="C27" s="20" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D27" s="21" t="n">
-        <v>14</v>
+        <v>150</v>
       </c>
       <c r="E27" s="21">
         <f>C27*D27</f>
@@ -5754,7 +5755,7 @@
       </c>
       <c r="F27" s="22" t="inlineStr">
         <is>
-          <t>SL63 / Gauze Pieces (Sterile)</t>
+          <t>SL87 / Moli / Mackintosh Sheet</t>
         </is>
       </c>
     </row>
@@ -5764,14 +5765,14 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Roller Bandage 6"</t>
+          <t>Inj. Neomol IV 10ml</t>
         </is>
       </c>
       <c r="C28" s="20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D28" s="21" t="n">
-        <v>67.5</v>
+        <v>42.8</v>
       </c>
       <c r="E28" s="21">
         <f>C28*D28</f>
@@ -5779,7 +5780,7 @@
       </c>
       <c r="F28" s="22" t="inlineStr">
         <is>
-          <t>SL74 / Roller Bandage 6" (Crepe)</t>
+          <t>SL28 / Inj. Neomol IV 10ml (PCM IV)</t>
         </is>
       </c>
     </row>
@@ -5789,14 +5790,14 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Betadine Lotion 100ml</t>
+          <t>Foley's Catheter 16 No.</t>
         </is>
       </c>
       <c r="C29" s="20" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="21" t="n">
-        <v>236.25</v>
+        <v>174</v>
       </c>
       <c r="E29" s="21">
         <f>C29*D29</f>
@@ -5804,7 +5805,7 @@
       </c>
       <c r="F29" s="22" t="inlineStr">
         <is>
-          <t>SL69 / Betadine Lotion 100ml</t>
+          <t>SL50 / Foley's Catheter 16 No.</t>
         </is>
       </c>
     </row>
@@ -5814,23 +5815,22 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Betadine Ointment 40g</t>
+          <t>Uro Bag</t>
         </is>
       </c>
       <c r="C30" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="23" t="inlineStr">
-        <is>
-          <t>⚠ ENTER MRP</t>
-        </is>
-      </c>
-      <c r="E30" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="25" t="inlineStr">
-        <is>
-          <t>SL71 — MRP missing, enter manually</t>
+      <c r="D30" s="21" t="n">
+        <v>361</v>
+      </c>
+      <c r="E30" s="21">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>SL49 / Uro Bag</t>
         </is>
       </c>
     </row>
@@ -5840,14 +5840,14 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Suture Ethilon 2-0</t>
+          <t>Inj. Ondem 2ml</t>
         </is>
       </c>
       <c r="C31" s="20" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D31" s="21" t="n">
-        <v>277</v>
+        <v>12.72</v>
       </c>
       <c r="E31" s="21">
         <f>C31*D31</f>
@@ -5855,7 +5855,7 @@
       </c>
       <c r="F31" s="22" t="inlineStr">
         <is>
-          <t>SL77 / Suture Ethilon 2-0 / SN9336TFP</t>
+          <t>SL29 / Inj. Ondem/Zofer/Zofar (Ondansetron</t>
         </is>
       </c>
     </row>
@@ -5865,14 +5865,14 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Suture Vicryl 1</t>
+          <t>Inj. Pan IV</t>
         </is>
       </c>
       <c r="C32" s="20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D32" s="21" t="n">
-        <v>250</v>
+        <v>53.9</v>
       </c>
       <c r="E32" s="21">
         <f>C32*D32</f>
@@ -5880,150 +5880,426 @@
       </c>
       <c r="F32" s="22" t="inlineStr">
         <is>
-          <t>SL78 / Suture Vicryl 1 (2421)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="26" t="inlineStr">
+          <t>SL33 / Inj. Pan 40 / Pantocid (Pantoprazol</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Xone 1g</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="E33" s="21">
+        <f>C33*D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>SL16 / Inj. Xone/Monocef 1g (Ceftriaxone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Diclofenac AQ (Justin)</t>
+        </is>
+      </c>
+      <c r="C34" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="21" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="E34" s="21">
+        <f>C34*D34</f>
+        <v/>
+      </c>
+      <c r="F34" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SL22 / Inj. Dynapar/Justin AQ (Diclofenac </t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Inj. PCM 100ml (Paracetamol IV)</t>
+        </is>
+      </c>
+      <c r="C35" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="21" t="n">
+        <v>591.3</v>
+      </c>
+      <c r="E35" s="21">
+        <f>C35*D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="22" t="inlineStr">
+        <is>
+          <t>SL27 / Inj. PCM 100ml (Paracetamol IV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Cetil (Cefuroxime Axetil)</t>
+        </is>
+      </c>
+      <c r="C36" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="21" t="n">
+        <v>346.9</v>
+      </c>
+      <c r="E36" s="21">
+        <f>C36*D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="22" t="inlineStr">
+        <is>
+          <t>SL21 / Inj. Cetil (Cefuroxime Axetil)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Tramadol 50mg</t>
+        </is>
+      </c>
+      <c r="C37" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="21" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="E37" s="21">
+        <f>C37*D37</f>
+        <v/>
+      </c>
+      <c r="F37" s="22" t="inlineStr">
+        <is>
+          <t>SL25 / Inj. Tramadol 50mg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Gloves 6.5 Sterile</t>
+        </is>
+      </c>
+      <c r="C38" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="21" t="n">
+        <v>97</v>
+      </c>
+      <c r="E38" s="21">
+        <f>C38*D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="22" t="inlineStr">
+        <is>
+          <t>SL66 / Gloves 6.5 (Sterile Surgical)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>Gauze Pieces (Sterile)</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="n">
+        <v>28</v>
+      </c>
+      <c r="D39" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="E39" s="21">
+        <f>C39*D39</f>
+        <v/>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>SL63 / Gauze Pieces (Sterile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Roller Bandage 6"</t>
+        </is>
+      </c>
+      <c r="C40" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="21" t="n">
+        <v>67.5</v>
+      </c>
+      <c r="E40" s="21">
+        <f>C40*D40</f>
+        <v/>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>SL74 / Roller Bandage 6" (Crepe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Gamji Roll</t>
+        </is>
+      </c>
+      <c r="C41" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="21" t="n">
+        <v>250</v>
+      </c>
+      <c r="E41" s="21">
+        <f>C41*D41</f>
+        <v/>
+      </c>
+      <c r="F41" s="22" t="inlineStr">
+        <is>
+          <t>SL108 / Gamji Roll</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Betadine Lotion 100ml</t>
+        </is>
+      </c>
+      <c r="C42" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="21" t="n">
+        <v>236.25</v>
+      </c>
+      <c r="E42" s="21">
+        <f>C42*D42</f>
+        <v/>
+      </c>
+      <c r="F42" s="22" t="inlineStr">
+        <is>
+          <t>SL69 / Betadine Lotion 100ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Betadine Ointment 40g</t>
+        </is>
+      </c>
+      <c r="C43" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>⚠ ENTER MRP</t>
+        </is>
+      </c>
+      <c r="E43" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="25" t="inlineStr">
+        <is>
+          <t>SL71 — MRP missing, enter manually</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="26" t="inlineStr">
         <is>
           <t>Consumables Sub-Total</t>
         </is>
       </c>
-      <c r="E33" s="27">
-        <f>SUMIF(E12:E32,"&gt;0",E12:E32)</f>
-        <v/>
-      </c>
-      <c r="F33" s="25" t="inlineStr">
-        <is>
-          <t>⚠ 1 item(s) need MRP — total partial</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="E44" s="27">
+        <f>SUMIF(E12:E43,"&gt;0",E12:E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="25" t="inlineStr">
+        <is>
+          <t>⚠ 2 item(s) need MRP — total partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>B.  BED CHARGES  +  C.  OT CHARGES</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Component</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>Rate (₹)</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Amount (₹)</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr"/>
-      <c r="F36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>Bed Charge (₹/day) — Bed Days in B8</t>
         </is>
       </c>
-      <c r="B37" s="21">
+      <c r="B48" s="21">
         <f>'RATES &amp; SUMMARY'!$B$4</f>
         <v/>
       </c>
-      <c r="C37" s="28">
+      <c r="C48" s="28">
         <f>B8</f>
         <v/>
       </c>
-      <c r="D37" s="29">
-        <f>B37*C37</f>
-        <v/>
-      </c>
-      <c r="E37" s="8" t="inlineStr"/>
-      <c r="F37" s="8" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="D48" s="29">
+        <f>B48*C48</f>
+        <v/>
+      </c>
+      <c r="E48" s="8" t="inlineStr"/>
+      <c r="F48" s="8" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>OT Charge (₹/hr) — OT Hours in B7</t>
         </is>
       </c>
-      <c r="B38" s="21">
+      <c r="B49" s="21">
         <f>'RATES &amp; SUMMARY'!$B$5</f>
         <v/>
       </c>
-      <c r="C38" s="28">
+      <c r="C49" s="28">
         <f>B7</f>
         <v/>
       </c>
-      <c r="D38" s="29">
-        <f>B38*C38</f>
-        <v/>
-      </c>
-      <c r="E38" s="8" t="inlineStr"/>
-      <c r="F38" s="8" t="inlineStr"/>
-    </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="30" t="inlineStr">
+      <c r="D49" s="29">
+        <f>B49*C49</f>
+        <v/>
+      </c>
+      <c r="E49" s="8" t="inlineStr"/>
+      <c r="F49" s="8" t="inlineStr"/>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="30" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="D40" s="31">
-        <f>E33+D37+D38</f>
-        <v/>
-      </c>
-      <c r="E40" s="32" t="inlineStr"/>
+      <c r="D51" s="31">
+        <f>E44+D48+D49</f>
+        <v/>
+      </c>
+      <c r="E51" s="32" t="inlineStr"/>
     </row>
     <row r="995">
       <c r="G995">
-        <f>E33+D37+D38</f>
+        <f>E44+D48+D49</f>
         <v/>
       </c>
     </row>
     <row r="996">
       <c r="G996">
-        <f>D38</f>
+        <f>D49</f>
         <v/>
       </c>
     </row>
     <row r="997">
       <c r="G997">
-        <f>D37</f>
+        <f>D48</f>
         <v/>
       </c>
     </row>
     <row r="999">
       <c r="E999">
-        <f>E33</f>
+        <f>E44</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="E51:F51"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="E40:F40"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A44:D44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Pt40 Rachel Hira bill: piles surgery OT sheet + ward indent (06/06/2026)
Items combined from OT consumable list (spinal, Dr. Rofik Ansari) and
Bed-1 ward indent: 22 line items, all priced from Master Rate Card.
Summary updated to 13 patients.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YWgR3jd3MUcEXpU4s4WC54
</commit_message>
<xml_diff>
--- a/BKAditya_June2026_Bills.xlsx
+++ b/BKAditya_June2026_Bills.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Pt37" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Pt38" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Pt39" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Pt40" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -166,7 +167,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -186,11 +187,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -281,6 +310,8 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -646,7 +677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -700,7 +731,7 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>PATIENT SUMMARY — ALL 12 BILLS  •  JUNE 2026</t>
+          <t>PATIENT SUMMARY — ALL 13 BILLS  •  JUNE 2026</t>
         </is>
       </c>
     </row>
@@ -1391,34 +1422,93 @@
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL — ALL 12 PATIENTS</t>
-        </is>
-      </c>
-      <c r="I21" s="13">
-        <f>SUM(I9:I20)</f>
-        <v/>
-      </c>
-      <c r="J21" s="13">
-        <f>SUM(J9:J20)</f>
-        <v/>
-      </c>
-      <c r="K21" s="13">
-        <f>SUM(K9:K20)</f>
-        <v/>
-      </c>
-      <c r="L21" s="13">
-        <f>SUM(L9:L20)</f>
+      <c r="A21" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Rachel Hira</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Dr. Rofik Ansari</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Piles Surgery</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Spinal</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="10">
+        <f>'Pt40'!E999</f>
+        <v/>
+      </c>
+      <c r="J21" s="10">
+        <f>'Pt40'!G997</f>
+        <v/>
+      </c>
+      <c r="K21" s="10">
+        <f>'Pt40'!G996</f>
+        <v/>
+      </c>
+      <c r="L21" s="11">
+        <f>'Pt40'!G995</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL — ALL 13 PATIENTS</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="n"/>
+      <c r="C22" s="34" t="n"/>
+      <c r="D22" s="34" t="n"/>
+      <c r="E22" s="34" t="n"/>
+      <c r="F22" s="34" t="n"/>
+      <c r="G22" s="34" t="n"/>
+      <c r="H22" s="35" t="n"/>
+      <c r="I22" s="13">
+        <f>SUM(I9:I21)</f>
+        <v/>
+      </c>
+      <c r="J22" s="13">
+        <f>SUM(J9:J21)</f>
+        <v/>
+      </c>
+      <c r="K22" s="13">
+        <f>SUM(K9:K21)</f>
+        <v/>
+      </c>
+      <c r="L22" s="13">
+        <f>SUM(L9:L21)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A7:K7"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1460,6 +1550,7 @@
           <t>Shyamal Santra</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -1472,6 +1563,7 @@
           <t>16/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -1484,6 +1576,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -1496,6 +1589,7 @@
           <t>TURP + Ward</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -1508,6 +1602,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -1518,6 +1613,7 @@
       <c r="B7" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -1528,6 +1624,7 @@
       <c r="B8" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -2101,6 +2198,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B33" s="34" t="n"/>
+      <c r="C33" s="34" t="n"/>
+      <c r="D33" s="35" t="n"/>
       <c r="E33" s="27">
         <f>SUMIF(E12:E32,"&gt;0",E12:E32)</f>
         <v/>
@@ -2190,11 +2290,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B40" s="34" t="n"/>
+      <c r="C40" s="35" t="n"/>
       <c r="D40" s="31">
         <f>E33+D37+D38</f>
         <v/>
       </c>
       <c r="E40" s="32" t="inlineStr"/>
+      <c r="F40" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -2276,6 +2379,7 @@
           <t>Md. Saiful Islam</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -2288,6 +2392,7 @@
           <t>18/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -2300,6 +2405,7 @@
           <t>Dr. K. Digga</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -2312,6 +2418,7 @@
           <t>Local OT + Ward</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -2324,6 +2431,7 @@
           <t>Local</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -2334,6 +2442,7 @@
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -2344,6 +2453,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -2716,6 +2826,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B25" s="34" t="n"/>
+      <c r="C25" s="34" t="n"/>
+      <c r="D25" s="35" t="n"/>
       <c r="E25" s="27">
         <f>SUMIF(E12:E24,"&gt;0",E12:E24)</f>
         <v/>
@@ -2805,11 +2918,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B32" s="34" t="n"/>
+      <c r="C32" s="35" t="n"/>
       <c r="D32" s="31">
         <f>E25+D29+D30</f>
         <v/>
       </c>
       <c r="E32" s="32" t="inlineStr"/>
+      <c r="F32" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -2891,6 +3007,7 @@
           <t>Depanita Sankar</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -2903,6 +3020,7 @@
           <t>21/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -2915,6 +3033,7 @@
           <t>Dr. K. Digga</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -2927,6 +3046,7 @@
           <t>Rt Femur Fracture Fixation + Ward</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -2939,6 +3059,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -2949,6 +3070,7 @@
       <c r="B7" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -2959,6 +3081,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -3356,6 +3479,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B26" s="34" t="n"/>
+      <c r="C26" s="34" t="n"/>
+      <c r="D26" s="35" t="n"/>
       <c r="E26" s="27">
         <f>SUMIF(E12:E25,"&gt;0",E12:E25)</f>
         <v/>
@@ -3445,11 +3571,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B33" s="34" t="n"/>
+      <c r="C33" s="35" t="n"/>
       <c r="D33" s="31">
         <f>E26+D30+D31</f>
         <v/>
       </c>
       <c r="E33" s="32" t="inlineStr"/>
+      <c r="F33" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -3479,8 +3608,8 @@
   <mergeCells count="13">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A28:F28"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="B3:C3"/>
@@ -3531,6 +3660,7 @@
           <t>MD Molla</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -3543,6 +3673,7 @@
           <t>22/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -3555,6 +3686,7 @@
           <t>Dr. K. Digga</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -3567,6 +3699,7 @@
           <t>Block OT + Ward</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -3579,6 +3712,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -3589,6 +3723,7 @@
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -3599,6 +3734,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -3870,6 +4006,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B21" s="34" t="n"/>
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="35" t="n"/>
       <c r="E21" s="27">
         <f>SUMIF(E12:E20,"&gt;0",E12:E20)</f>
         <v/>
@@ -3959,11 +4098,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="35" t="n"/>
       <c r="D28" s="31">
         <f>E21+D25+D26</f>
         <v/>
       </c>
       <c r="E28" s="32" t="inlineStr"/>
+      <c r="F28" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -4002,6 +4144,852 @@
     <mergeCell ref="A23:F23"/>
     <mergeCell ref="A21:D21"/>
     <mergeCell ref="E28:F28"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G999"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="1" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>BK ADITYA MULTISPECIALTY HOSPITAL — PATIENT BILL  #40</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Patient Name</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Rachel Hira</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Doctor</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Dr. Rofik Ansari</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Procedure</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Piles Surgery</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Anaesthesia</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Spinal</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>OT Hours</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="35" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Bed Days</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="35" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>A.  CONSUMABLES / MEDICINES</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Item Description</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Rate (MRP ₹)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Amount (₹)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Spinal Needle 25G (Spinocaine)</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>153</v>
+      </c>
+      <c r="E12" s="21">
+        <f>C12*D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>SL55 / Spinal Needle 25G (Spinocan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Anawin Heavy 0.75%</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>31.47</v>
+      </c>
+      <c r="E13" s="21">
+        <f>C13*D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>SL7 / Inj. Anawin Heavy 0.75%/4ml (Bupiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Pause 500mg</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>71.97</v>
+      </c>
+      <c r="E14" s="21">
+        <f>C14*D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>SL40 / Inj. Pause 500mg (Tranexamic Acid)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>D. Water 10ml</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="21" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E15" s="21">
+        <f>C15*D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>SL59 / D. Water 10ml (Sterile Water)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Gauze Pieces (Sterile)</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="21" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="21">
+        <f>C16*D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>SL63 / Gauze Pieces (Sterile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Plain Sheet (OT)</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="21" t="n">
+        <v>200</v>
+      </c>
+      <c r="E17" s="21">
+        <f>C17*D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>SL83 / Plain Sheet (OT Draping)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Gloves 7.0 Sterile</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>91</v>
+      </c>
+      <c r="E18" s="21">
+        <f>C18*D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>SL65 / Gloves 7.0 (Sterile Surgical)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Gloves 6.5 Sterile</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>97</v>
+      </c>
+      <c r="E19" s="21">
+        <f>C19*D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>SL66 / Gloves 6.5 (Sterile Surgical)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Betadine Lotion 100ml</t>
+        </is>
+      </c>
+      <c r="C20" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>236.25</v>
+      </c>
+      <c r="E20" s="21">
+        <f>C20*D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>SL69 / Betadine Lotion 100ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>RL 500ml</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="E21" s="21">
+        <f>C21*D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>SL4 / RL 500ml — Ringer's Lactate</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>NS 500ml</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>39.05</v>
+      </c>
+      <c r="E22" s="21">
+        <f>C22*D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>SL1 / NS 500ml — OT ×1 + Ward ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Rantac 2ml</t>
+        </is>
+      </c>
+      <c r="C23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="E23" s="21">
+        <f>C23*D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>SL30 / Inj. Rantac (Ranitidine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Ondem 2ml</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="21" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="E24" s="21">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>SL29 / Inj. Ondem/Zofer/Zofar (Ondansetron</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Xone 1g</t>
+        </is>
+      </c>
+      <c r="C25" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" s="21" t="n">
+        <v>66.64</v>
+      </c>
+      <c r="E25" s="21">
+        <f>C25*D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>SL16 / Inj. Xone/Monocef 1g (Ceftriaxone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Metrogyl 100ml</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="21" t="n">
+        <v>22.05</v>
+      </c>
+      <c r="E26" s="21">
+        <f>C26*D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SL20 / Inj. Metrogyl 100ml (Metronidazole </t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Inj. Dynapar AQ 2ml</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="21" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="E27" s="21">
+        <f>C27*D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SL22 / Inj. Dynapar/Justin AQ (Diclofenac </t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Syringe 10ml</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" s="21">
+        <f>C28*D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>SL56 / Syringe 10cc — OT ×1 + Ward ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Syringe 5ml</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="21" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="E29" s="21">
+        <f>C29*D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>SL57 / Syringe 5cc — OT ×1 + Ward ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Syringe 2ml</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="21" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="E30" s="21">
+        <f>C30*D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>SL58 / Syringe 2cc / 2ml</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>IV Cannula 18G</t>
+        </is>
+      </c>
+      <c r="C31" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="21" t="n">
+        <v>321</v>
+      </c>
+      <c r="E31" s="21">
+        <f>C31*D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>SL47 / IV Cannula 18G / Venflon 18G</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Easyfix</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="21" t="n">
+        <v>900</v>
+      </c>
+      <c r="E32" s="21">
+        <f>C32*D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>SL48 / Easyfix (Adhesive Film Dressing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>IV Set</t>
+        </is>
+      </c>
+      <c r="C33" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>201</v>
+      </c>
+      <c r="E33" s="21">
+        <f>C33*D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>SL44 / IV Set / Sangoflex</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="26" t="inlineStr">
+        <is>
+          <t>Consumables Sub-Total</t>
+        </is>
+      </c>
+      <c r="B34" s="34" t="n"/>
+      <c r="C34" s="34" t="n"/>
+      <c r="D34" s="35" t="n"/>
+      <c r="E34" s="27">
+        <f>SUMIF(E12:E33,"&gt;0",E12:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="25" t="inlineStr">
+        <is>
+          <t>All items priced from Master Rate Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>B.  BED CHARGES  +  C.  OT CHARGES</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Rate (₹)</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Amount (₹)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Bed Charge (₹/day) — Bed Days in B8</t>
+        </is>
+      </c>
+      <c r="B38" s="21">
+        <f>'RATES &amp; SUMMARY'!$B$4</f>
+        <v/>
+      </c>
+      <c r="C38" s="28">
+        <f>B8</f>
+        <v/>
+      </c>
+      <c r="D38" s="29">
+        <f>B38*C38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>OT Charge (₹/hr) — OT Hours in B7</t>
+        </is>
+      </c>
+      <c r="B39" s="21">
+        <f>'RATES &amp; SUMMARY'!$B$5</f>
+        <v/>
+      </c>
+      <c r="C39" s="28">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="D39" s="29">
+        <f>B39*C39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B41" s="34" t="n"/>
+      <c r="C41" s="35" t="n"/>
+      <c r="D41" s="31">
+        <f>E34+D38+D39</f>
+        <v/>
+      </c>
+      <c r="E41" s="32" t="n"/>
+      <c r="F41" s="35" t="n"/>
+    </row>
+    <row r="995">
+      <c r="G995">
+        <f>E34+D38+D39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="996">
+      <c r="G996">
+        <f>D39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="997">
+      <c r="G997">
+        <f>D38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="999">
+      <c r="E999">
+        <f>E34</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="E41:F41"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
@@ -4045,6 +5033,7 @@
           <t>Prabir Kumar Paul</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -4057,6 +5046,7 @@
           <t>02/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -4069,6 +5059,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -4081,6 +5072,7 @@
           <t>Excision Biopsy</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -4093,6 +5085,7 @@
           <t>Local</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -4103,6 +5096,7 @@
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -4113,6 +5107,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -4435,6 +5430,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B23" s="34" t="n"/>
+      <c r="C23" s="34" t="n"/>
+      <c r="D23" s="35" t="n"/>
       <c r="E23" s="27">
         <f>SUMIF(E12:E22,"&gt;0",E12:E22)</f>
         <v/>
@@ -4524,11 +5522,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="35" t="n"/>
       <c r="D30" s="31">
         <f>E23+D27+D28</f>
         <v/>
       </c>
       <c r="E30" s="32" t="inlineStr"/>
+      <c r="F30" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -4610,6 +5611,7 @@
           <t>Sopna</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -4622,6 +5624,7 @@
           <t>08/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -4634,6 +5637,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -4646,6 +5650,7 @@
           <t>PIRS Spine Surgery</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -4658,6 +5663,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -4668,6 +5674,7 @@
       <c r="B7" s="18" t="n">
         <v>4</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -4678,6 +5685,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -5075,6 +6083,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B26" s="34" t="n"/>
+      <c r="C26" s="34" t="n"/>
+      <c r="D26" s="35" t="n"/>
       <c r="E26" s="27">
         <f>SUMIF(E12:E25,"&gt;0",E12:E25)</f>
         <v/>
@@ -5164,11 +6175,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B33" s="34" t="n"/>
+      <c r="C33" s="35" t="n"/>
       <c r="D33" s="31">
         <f>E26+D30+D31</f>
         <v/>
       </c>
       <c r="E33" s="32" t="inlineStr"/>
+      <c r="F33" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -5198,8 +6212,8 @@
   <mergeCells count="13">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A28:F28"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="B3:C3"/>
@@ -5250,6 +6264,7 @@
           <t>Shankari Chakraborty</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -5262,6 +6277,7 @@
           <t>08/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -5274,6 +6290,7 @@
           <t>Dr. K. Digga</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -5286,6 +6303,7 @@
           <t>Total Knee Replacement (TKR)</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -5298,6 +6316,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -5308,6 +6327,7 @@
       <c r="B7" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -5318,6 +6338,7 @@
       <c r="B8" s="18" t="n">
         <v>6</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -6166,6 +7187,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B44" s="34" t="n"/>
+      <c r="C44" s="34" t="n"/>
+      <c r="D44" s="35" t="n"/>
       <c r="E44" s="27">
         <f>SUMIF(E12:E43,"&gt;0",E12:E43)</f>
         <v/>
@@ -6255,11 +7279,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B51" s="34" t="n"/>
+      <c r="C51" s="35" t="n"/>
       <c r="D51" s="31">
         <f>E44+D48+D49</f>
         <v/>
       </c>
       <c r="E51" s="32" t="inlineStr"/>
+      <c r="F51" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -6341,6 +7368,7 @@
           <t>Kalipada Mondal</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -6353,6 +7381,7 @@
           <t>09/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -6365,6 +7394,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -6377,6 +7407,7 @@
           <t>TURP</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -6389,6 +7420,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -6399,6 +7431,7 @@
       <c r="B7" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -6409,6 +7442,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -6955,6 +7989,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B32" s="34" t="n"/>
+      <c r="C32" s="34" t="n"/>
+      <c r="D32" s="35" t="n"/>
       <c r="E32" s="27">
         <f>SUMIF(E12:E31,"&gt;0",E12:E31)</f>
         <v/>
@@ -7044,11 +8081,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B39" s="34" t="n"/>
+      <c r="C39" s="35" t="n"/>
       <c r="D39" s="31">
         <f>E32+D36+D37</f>
         <v/>
       </c>
       <c r="E39" s="32" t="inlineStr"/>
+      <c r="F39" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -7130,6 +8170,7 @@
           <t>Ripusudan Sankar</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -7142,6 +8183,7 @@
           <t>09/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -7154,6 +8196,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -7166,6 +8209,7 @@
           <t>Cystoscopy</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -7178,6 +8222,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -7188,6 +8233,7 @@
       <c r="B7" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -7198,6 +8244,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -7419,6 +8466,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B19" s="34" t="n"/>
+      <c r="C19" s="34" t="n"/>
+      <c r="D19" s="35" t="n"/>
       <c r="E19" s="27">
         <f>SUMIF(E12:E18,"&gt;0",E12:E18)</f>
         <v/>
@@ -7508,11 +8558,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B26" s="34" t="n"/>
+      <c r="C26" s="35" t="n"/>
       <c r="D26" s="31">
         <f>E19+D23+D24</f>
         <v/>
       </c>
       <c r="E26" s="32" t="inlineStr"/>
+      <c r="F26" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -7547,11 +8600,11 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="E26:F26"/>
-    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="A21:F21"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A26:C26"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7594,6 +8647,7 @@
           <t>Sahid Ali Joddar</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -7606,6 +8660,7 @@
           <t>12/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -7618,6 +8673,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -7630,6 +8686,7 @@
           <t>TWA</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -7642,6 +8699,7 @@
           <t>General</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -7652,6 +8710,7 @@
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -7662,6 +8721,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -7858,6 +8918,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B18" s="34" t="n"/>
+      <c r="C18" s="34" t="n"/>
+      <c r="D18" s="35" t="n"/>
       <c r="E18" s="27">
         <f>SUMIF(E12:E17,"&gt;0",E12:E17)</f>
         <v/>
@@ -7947,11 +9010,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B25" s="34" t="n"/>
+      <c r="C25" s="35" t="n"/>
       <c r="D25" s="31">
         <f>E18+D22+D23</f>
         <v/>
       </c>
       <c r="E25" s="32" t="inlineStr"/>
+      <c r="F25" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -8033,6 +9099,7 @@
           <t>Khogen Naskar</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -8045,6 +9112,7 @@
           <t>12/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -8057,6 +9125,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -8069,6 +9138,7 @@
           <t>Cystoscopy</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -8081,6 +9151,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -8091,6 +9162,7 @@
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -8101,6 +9173,7 @@
       <c r="B8" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -8398,6 +9471,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B22" s="34" t="n"/>
+      <c r="C22" s="34" t="n"/>
+      <c r="D22" s="35" t="n"/>
       <c r="E22" s="27">
         <f>SUMIF(E12:E21,"&gt;0",E12:E21)</f>
         <v/>
@@ -8487,11 +9563,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="35" t="n"/>
       <c r="D29" s="31">
         <f>E22+D26+D27</f>
         <v/>
       </c>
       <c r="E29" s="32" t="inlineStr"/>
+      <c r="F29" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">
@@ -8573,6 +9652,7 @@
           <t>Rahima Bibi Malla</t>
         </is>
       </c>
+      <c r="C2" s="35" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -8585,6 +9665,7 @@
           <t>15/06/2026</t>
         </is>
       </c>
+      <c r="C3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
@@ -8597,6 +9678,7 @@
           <t>Dr. S. Gupta</t>
         </is>
       </c>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
@@ -8609,6 +9691,7 @@
           <t>STG (OT) + Ward</t>
         </is>
       </c>
+      <c r="C5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
@@ -8621,6 +9704,7 @@
           <t>Spinal</t>
         </is>
       </c>
+      <c r="C6" s="35" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
@@ -8631,6 +9715,7 @@
       <c r="B7" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
@@ -8641,6 +9726,7 @@
       <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -9463,6 +10549,9 @@
           <t>Consumables Sub-Total</t>
         </is>
       </c>
+      <c r="B43" s="34" t="n"/>
+      <c r="C43" s="34" t="n"/>
+      <c r="D43" s="35" t="n"/>
       <c r="E43" s="27">
         <f>SUMIF(E12:E42,"&gt;0",E12:E42)</f>
         <v/>
@@ -9552,11 +10641,14 @@
           <t>GRAND TOTAL</t>
         </is>
       </c>
+      <c r="B50" s="34" t="n"/>
+      <c r="C50" s="35" t="n"/>
       <c r="D50" s="31">
         <f>E43+D47+D48</f>
         <v/>
       </c>
       <c r="E50" s="32" t="inlineStr"/>
+      <c r="F50" s="35" t="n"/>
     </row>
     <row r="995">
       <c r="G995">

</xml_diff>